<commit_message>
Update clinical and standard data Excel files
Replaced standard_data.xlsx with standard_data_v4.xlsx and updated emr_clinical_data_component.xlsx. These changes likely reflect updates to the data structure or content in the Excel files.
</commit_message>
<xml_diff>
--- a/emr_clinical_data_component.xlsx
+++ b/emr_clinical_data_component.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GoogleDrive\nkakada\NPCA\workshop\20251016_api_hospital\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\npcai\Herd\emr-standards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB229FFF-F741-4D97-8356-A6A41BE0F68E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85D5713-318E-4123-B513-C33795AC5C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="API Objects" sheetId="1" r:id="rId1"/>
@@ -1094,7 +1094,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1192,6 +1192,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1200,9 +1203,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1723,27 +1723,27 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G251"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="23.25" x14ac:dyDescent="0.65"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="23.25"/>
   <cols>
-    <col min="1" max="1" width="28.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="59.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.42578125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="62.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="28.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="59.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="62.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="29.25" x14ac:dyDescent="0.8">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:5" ht="29.25">
+      <c r="A1" s="9" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.65">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1760,7 +1760,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1777,7 +1777,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="4" spans="1:5">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
         <v>8</v>
@@ -1792,7 +1792,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="5" spans="1:5">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
         <v>10</v>
@@ -1807,7 +1807,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="6" spans="1:5">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
         <v>12</v>
@@ -1822,7 +1822,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="7" spans="1:5">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
         <v>14</v>
@@ -1837,7 +1837,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="8" spans="1:5">
       <c r="A8" s="2"/>
       <c r="B8" s="2" t="s">
         <v>17</v>
@@ -1852,7 +1852,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="9" spans="1:5">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
         <v>283</v>
@@ -1867,7 +1867,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="10" spans="1:5">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
         <v>18</v>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="11" spans="1:5">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
         <v>20</v>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="12" spans="1:5">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
         <v>22</v>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="13" spans="1:5">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
         <v>24</v>
@@ -1919,7 +1919,7 @@
       </c>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="14" spans="1:5">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
         <v>25</v>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="15" spans="1:5">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
         <v>286</v>
@@ -1947,7 +1947,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="16" spans="1:5">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
         <v>28</v>
@@ -1962,7 +1962,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="17" spans="1:5">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
         <v>30</v>
@@ -1977,7 +1977,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="18" spans="1:5">
       <c r="A18" s="3" t="s">
         <v>32</v>
       </c>
@@ -1994,7 +1994,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="19" spans="1:5">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
         <v>35</v>
@@ -2009,7 +2009,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="20" spans="1:5">
       <c r="A20" s="2"/>
       <c r="B20" s="2" t="s">
         <v>36</v>
@@ -2024,7 +2024,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="21" spans="1:5">
       <c r="A21" s="2"/>
       <c r="B21" s="2" t="s">
         <v>38</v>
@@ -2039,7 +2039,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="22" spans="1:5">
       <c r="A22" s="2"/>
       <c r="B22" s="2" t="s">
         <v>39</v>
@@ -2054,7 +2054,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="23" spans="1:5">
       <c r="A23" s="2"/>
       <c r="B23" s="2" t="s">
         <v>41</v>
@@ -2069,7 +2069,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="24" spans="1:5">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
         <v>42</v>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="25" spans="1:5">
       <c r="A25" s="2"/>
       <c r="B25" s="2" t="s">
         <v>44</v>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="26" spans="1:5">
       <c r="A26" s="2"/>
       <c r="B26" s="2" t="s">
         <v>45</v>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="27" spans="1:5">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
         <v>47</v>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="E27" s="2"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="28" spans="1:5">
       <c r="A28" s="2"/>
       <c r="B28" s="2" t="s">
         <v>49</v>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="29" spans="1:5">
       <c r="A29" s="3" t="s">
         <v>255</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="30" spans="1:5">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
         <v>53</v>
@@ -2166,7 +2166,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="31" spans="1:5">
       <c r="A31" s="2"/>
       <c r="B31" s="2" t="s">
         <v>313</v>
@@ -2181,7 +2181,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="32" spans="1:5">
       <c r="A32" s="3" t="s">
         <v>56</v>
       </c>
@@ -2198,7 +2198,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="33" spans="1:5">
       <c r="A33" s="2"/>
       <c r="B33" s="2" t="s">
         <v>51</v>
@@ -2213,7 +2213,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="34" spans="1:5">
       <c r="A34" s="2"/>
       <c r="B34" s="2" t="s">
         <v>5</v>
@@ -2228,7 +2228,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="35" spans="1:5">
       <c r="A35" s="2"/>
       <c r="B35" s="2" t="s">
         <v>314</v>
@@ -2243,7 +2243,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="36" spans="1:5">
       <c r="A36" s="2"/>
       <c r="B36" s="2" t="s">
         <v>315</v>
@@ -2258,7 +2258,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="37" spans="1:5">
       <c r="A37" s="2"/>
       <c r="B37" s="2" t="s">
         <v>316</v>
@@ -2273,7 +2273,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="38" spans="1:5">
       <c r="A38" s="2"/>
       <c r="B38" s="2" t="s">
         <v>317</v>
@@ -2288,7 +2288,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="39" spans="1:5">
       <c r="A39" s="2"/>
       <c r="B39" s="2" t="s">
         <v>60</v>
@@ -2303,7 +2303,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="40" spans="1:5">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
         <v>62</v>
@@ -2318,7 +2318,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="41" spans="1:5">
       <c r="A41" s="2"/>
       <c r="B41" s="2" t="s">
         <v>64</v>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="E41" s="2"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="42" spans="1:5">
       <c r="A42" s="2"/>
       <c r="B42" s="2" t="s">
         <v>28</v>
@@ -2346,7 +2346,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="43" spans="1:5">
       <c r="A43" s="2"/>
       <c r="B43" s="2" t="s">
         <v>30</v>
@@ -2361,7 +2361,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="44" spans="1:5">
       <c r="A44" s="3" t="s">
         <v>83</v>
       </c>
@@ -2378,7 +2378,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="45" spans="1:5">
       <c r="A45" s="3"/>
       <c r="B45" s="2" t="s">
         <v>65</v>
@@ -2393,7 +2393,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="46" spans="1:5">
       <c r="A46" s="3"/>
       <c r="B46" s="2" t="s">
         <v>74</v>
@@ -2408,7 +2408,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="47" spans="1:5">
       <c r="A47" s="2"/>
       <c r="B47" s="2" t="s">
         <v>5</v>
@@ -2423,7 +2423,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="48" spans="1:5">
       <c r="A48" s="2"/>
       <c r="B48" s="2" t="s">
         <v>85</v>
@@ -2438,7 +2438,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="49" spans="1:5">
       <c r="A49" s="2"/>
       <c r="B49" s="2" t="s">
         <v>88</v>
@@ -2453,7 +2453,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="50" spans="1:5">
       <c r="A50" s="2"/>
       <c r="B50" s="2" t="s">
         <v>91</v>
@@ -2468,7 +2468,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="51" spans="1:5">
       <c r="A51" s="2"/>
       <c r="B51" s="2" t="s">
         <v>93</v>
@@ -2483,7 +2483,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="52" spans="1:5">
       <c r="A52" s="2"/>
       <c r="B52" s="2" t="s">
         <v>95</v>
@@ -2498,7 +2498,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="53" spans="1:5">
       <c r="A53" s="2"/>
       <c r="B53" s="2" t="s">
         <v>318</v>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="E53" s="2"/>
     </row>
-    <row r="54" spans="1:5" ht="46.5" x14ac:dyDescent="0.65">
+    <row r="54" spans="1:5" ht="46.5">
       <c r="A54" s="3" t="s">
         <v>267</v>
       </c>
@@ -2528,7 +2528,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="55" spans="1:5">
       <c r="A55" s="2"/>
       <c r="B55" s="2" t="s">
         <v>93</v>
@@ -2543,7 +2543,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="56" spans="1:5">
       <c r="A56" s="2"/>
       <c r="B56" s="2" t="s">
         <v>95</v>
@@ -2558,7 +2558,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="57" spans="1:5">
       <c r="A57" s="2"/>
       <c r="B57" s="2" t="s">
         <v>318</v>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="E57" s="2"/>
     </row>
-    <row r="58" spans="1:5" ht="76.5" customHeight="1" x14ac:dyDescent="0.65">
+    <row r="58" spans="1:5" ht="76.5" customHeight="1">
       <c r="A58" s="3" t="s">
         <v>266</v>
       </c>
@@ -2588,7 +2588,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="59" spans="1:5">
       <c r="A59" s="2"/>
       <c r="B59" s="2" t="s">
         <v>78</v>
@@ -2603,7 +2603,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="60" spans="1:5">
       <c r="A60" s="3" t="s">
         <v>265</v>
       </c>
@@ -2620,7 +2620,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="61" spans="1:5">
       <c r="A61" s="3"/>
       <c r="B61" s="2" t="s">
         <v>65</v>
@@ -2635,7 +2635,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="62" spans="1:5">
       <c r="A62" s="3"/>
       <c r="B62" s="2" t="s">
         <v>74</v>
@@ -2650,7 +2650,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="63" spans="1:5">
       <c r="A63" s="2"/>
       <c r="B63" s="2" t="s">
         <v>10</v>
@@ -2665,7 +2665,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="64" spans="1:5">
       <c r="A64" s="2"/>
       <c r="B64" s="2" t="s">
         <v>78</v>
@@ -2680,7 +2680,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="65" spans="1:7">
       <c r="A65" s="3" t="s">
         <v>105</v>
       </c>
@@ -2697,7 +2697,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="66" spans="1:7">
       <c r="A66" s="3"/>
       <c r="B66" s="2" t="s">
         <v>65</v>
@@ -2712,7 +2712,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="67" spans="1:7">
       <c r="A67" s="3"/>
       <c r="B67" s="2" t="s">
         <v>74</v>
@@ -2727,7 +2727,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="68" spans="1:7">
       <c r="A68" s="2"/>
       <c r="B68" s="2" t="s">
         <v>10</v>
@@ -2742,7 +2742,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="69" spans="1:7">
       <c r="A69" s="2"/>
       <c r="B69" s="2" t="s">
         <v>78</v>
@@ -2757,7 +2757,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="70" spans="1:7">
       <c r="A70" s="2"/>
       <c r="B70" s="2" t="s">
         <v>80</v>
@@ -2772,7 +2772,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="71" spans="1:7">
       <c r="A71" s="2"/>
       <c r="B71" s="2" t="s">
         <v>81</v>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="E71" s="2"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="72" spans="1:7">
       <c r="A72" s="3" t="s">
         <v>259</v>
       </c>
@@ -2802,7 +2802,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="73" spans="1:7">
       <c r="A73" s="3"/>
       <c r="B73" s="2" t="s">
         <v>65</v>
@@ -2817,7 +2817,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="74" spans="1:7">
       <c r="A74" s="3"/>
       <c r="B74" s="2" t="s">
         <v>74</v>
@@ -2832,7 +2832,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="75" spans="1:7">
       <c r="A75" s="3"/>
       <c r="B75" s="2" t="s">
         <v>5</v>
@@ -2847,7 +2847,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="76" spans="1:7">
       <c r="A76" s="2"/>
       <c r="B76" s="2" t="s">
         <v>272</v>
@@ -2862,7 +2862,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="77" spans="1:7">
       <c r="A77" s="3"/>
       <c r="B77" s="2" t="s">
         <v>273</v>
@@ -2877,7 +2877,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="78" spans="1:7">
       <c r="A78" s="3"/>
       <c r="B78" s="2" t="s">
         <v>318</v>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="E78" s="2"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.65">
+    <row r="79" spans="1:7">
       <c r="A79" s="3" t="s">
         <v>277</v>
       </c>
@@ -2906,10 +2906,10 @@
       <c r="E79" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F79" s="9"/>
-      <c r="G79" s="9"/>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.65">
+      <c r="F79" s="10"/>
+      <c r="G79" s="10"/>
+    </row>
+    <row r="80" spans="1:7">
       <c r="A80" s="2"/>
       <c r="B80" s="2" t="s">
         <v>10</v>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="F80" s="7"/>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="81" spans="1:5">
       <c r="A81" s="2"/>
       <c r="B81" s="2" t="s">
         <v>77</v>
@@ -2940,7 +2940,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="82" spans="1:5">
       <c r="A82" s="2"/>
       <c r="B82" s="2" t="s">
         <v>78</v>
@@ -2955,7 +2955,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="83" spans="1:5">
       <c r="A83" s="2"/>
       <c r="B83" s="2" t="s">
         <v>80</v>
@@ -2970,7 +2970,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="84" spans="1:5">
       <c r="A84" s="2"/>
       <c r="B84" s="2" t="s">
         <v>81</v>
@@ -2985,7 +2985,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="85" spans="1:5">
       <c r="A85" s="2"/>
       <c r="B85" s="2" t="s">
         <v>121</v>
@@ -3000,7 +3000,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="86" spans="1:5">
       <c r="A86" s="2"/>
       <c r="B86" s="2" t="s">
         <v>123</v>
@@ -3015,7 +3015,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="87" spans="1:5">
       <c r="A87" s="2"/>
       <c r="B87" s="2" t="s">
         <v>322</v>
@@ -3030,7 +3030,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="88" spans="1:5">
       <c r="A88" s="2"/>
       <c r="B88" s="2" t="s">
         <v>323</v>
@@ -3045,7 +3045,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="89" spans="1:5">
       <c r="A89" s="2"/>
       <c r="B89" s="2" t="s">
         <v>93</v>
@@ -3060,7 +3060,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="90" spans="1:5">
       <c r="A90" s="2"/>
       <c r="B90" s="2" t="s">
         <v>95</v>
@@ -3075,7 +3075,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="91" spans="1:5">
       <c r="A91" s="3" t="s">
         <v>258</v>
       </c>
@@ -3092,7 +3092,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="92" spans="1:5">
       <c r="A92" s="3"/>
       <c r="B92" s="2" t="s">
         <v>65</v>
@@ -3107,7 +3107,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="93" spans="1:5">
       <c r="A93" s="3"/>
       <c r="B93" s="2" t="s">
         <v>74</v>
@@ -3122,7 +3122,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="94" spans="1:5">
       <c r="A94" s="3"/>
       <c r="B94" s="2" t="s">
         <v>312</v>
@@ -3137,7 +3137,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="95" spans="1:5">
       <c r="A95" s="2"/>
       <c r="B95" s="2" t="s">
         <v>272</v>
@@ -3152,7 +3152,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="96" spans="1:5">
       <c r="A96" s="3"/>
       <c r="B96" s="2" t="s">
         <v>273</v>
@@ -3167,7 +3167,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="97" spans="1:5">
       <c r="A97" s="3"/>
       <c r="B97" s="2" t="s">
         <v>318</v>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="E97" s="2"/>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="98" spans="1:5">
       <c r="A98" s="3" t="s">
         <v>271</v>
       </c>
@@ -3197,7 +3197,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="99" spans="1:5">
       <c r="A99" s="2"/>
       <c r="B99" s="2" t="s">
         <v>77</v>
@@ -3212,7 +3212,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="100" spans="1:5">
       <c r="A100" s="2"/>
       <c r="B100" s="2" t="s">
         <v>127</v>
@@ -3227,7 +3227,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="101" spans="1:5">
       <c r="A101" s="2"/>
       <c r="B101" s="2" t="s">
         <v>129</v>
@@ -3242,7 +3242,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="102" spans="1:5">
       <c r="A102" s="2"/>
       <c r="B102" s="2" t="s">
         <v>296</v>
@@ -3257,7 +3257,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="103" spans="1:5">
       <c r="A103" s="2"/>
       <c r="B103" s="2" t="s">
         <v>322</v>
@@ -3272,7 +3272,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="104" spans="1:5">
       <c r="A104" s="2"/>
       <c r="B104" s="2" t="s">
         <v>323</v>
@@ -3287,7 +3287,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="105" spans="1:5">
       <c r="A105" s="2"/>
       <c r="B105" s="2" t="s">
         <v>93</v>
@@ -3302,7 +3302,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="106" spans="1:5">
       <c r="A106" s="2"/>
       <c r="B106" s="2" t="s">
         <v>95</v>
@@ -3317,7 +3317,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="107" spans="1:5">
       <c r="A107" s="3" t="s">
         <v>268</v>
       </c>
@@ -3334,7 +3334,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="108" spans="1:5">
       <c r="A108" s="3"/>
       <c r="B108" s="2" t="s">
         <v>65</v>
@@ -3349,7 +3349,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="109" spans="1:5">
       <c r="A109" s="2"/>
       <c r="B109" s="2" t="s">
         <v>74</v>
@@ -3364,7 +3364,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="110" spans="1:5">
       <c r="A110" s="2"/>
       <c r="B110" s="2" t="s">
         <v>109</v>
@@ -3379,7 +3379,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="111" spans="1:5">
       <c r="A111" s="2"/>
       <c r="B111" s="2" t="s">
         <v>110</v>
@@ -3394,7 +3394,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="112" spans="1:5">
       <c r="A112" s="2"/>
       <c r="B112" s="2" t="s">
         <v>112</v>
@@ -3409,7 +3409,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="113" spans="1:6">
       <c r="A113" s="2"/>
       <c r="B113" s="2" t="s">
         <v>114</v>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="E113" s="2"/>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="114" spans="1:6">
       <c r="A114" s="2"/>
       <c r="B114" s="2" t="s">
         <v>115</v>
@@ -3437,7 +3437,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="115" spans="1:6">
       <c r="A115" s="2"/>
       <c r="B115" s="2" t="s">
         <v>117</v>
@@ -3452,7 +3452,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="116" spans="1:6">
       <c r="A116" s="2"/>
       <c r="B116" s="2" t="s">
         <v>318</v>
@@ -3465,7 +3465,7 @@
       </c>
       <c r="E116" s="2"/>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="117" spans="1:6">
       <c r="A117" s="3" t="s">
         <v>264</v>
       </c>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="E117" s="2"/>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="118" spans="1:6">
       <c r="A118" s="3"/>
       <c r="B118" s="2" t="s">
         <v>247</v>
@@ -3493,7 +3493,7 @@
       </c>
       <c r="E118" s="2"/>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="119" spans="1:6">
       <c r="A119" s="2"/>
       <c r="B119" s="2" t="s">
         <v>249</v>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="E119" s="2"/>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="120" spans="1:6">
       <c r="A120" s="2"/>
       <c r="B120" s="2" t="s">
         <v>251</v>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="E120" s="2"/>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="121" spans="1:6">
       <c r="A121" s="2"/>
       <c r="B121" s="2" t="s">
         <v>326</v>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="E121" s="2"/>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="122" spans="1:6">
       <c r="A122" s="2"/>
       <c r="B122" s="2" t="s">
         <v>253</v>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="E122" s="2"/>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="123" spans="1:6">
       <c r="A123" s="3" t="s">
         <v>260</v>
       </c>
@@ -3561,11 +3561,11 @@
       <c r="E123" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F123" s="10" t="s">
+      <c r="F123" s="11" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="124" spans="1:6">
       <c r="A124" s="3"/>
       <c r="B124" s="2" t="s">
         <v>65</v>
@@ -3579,9 +3579,9 @@
       <c r="E124" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F124" s="10"/>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F124" s="11"/>
+    </row>
+    <row r="125" spans="1:6">
       <c r="A125" s="3"/>
       <c r="B125" s="2" t="s">
         <v>74</v>
@@ -3595,9 +3595,9 @@
       <c r="E125" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="F125" s="10"/>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F125" s="11"/>
+    </row>
+    <row r="126" spans="1:6">
       <c r="A126" s="2"/>
       <c r="B126" s="2" t="s">
         <v>5</v>
@@ -3611,9 +3611,9 @@
       <c r="E126" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F126" s="10"/>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F126" s="11"/>
+    </row>
+    <row r="127" spans="1:6">
       <c r="A127" s="2"/>
       <c r="B127" s="2" t="s">
         <v>133</v>
@@ -3627,9 +3627,9 @@
       <c r="E127" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F127" s="10"/>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F127" s="11"/>
+    </row>
+    <row r="128" spans="1:6">
       <c r="A128" s="2"/>
       <c r="B128" s="2" t="s">
         <v>135</v>
@@ -3643,9 +3643,9 @@
       <c r="E128" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F128" s="10"/>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F128" s="11"/>
+    </row>
+    <row r="129" spans="1:6">
       <c r="A129" s="2"/>
       <c r="B129" s="2" t="s">
         <v>318</v>
@@ -3657,9 +3657,9 @@
         <v>328</v>
       </c>
       <c r="E129" s="2"/>
-      <c r="F129" s="10"/>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F129" s="11"/>
+    </row>
+    <row r="130" spans="1:6">
       <c r="A130" s="3" t="s">
         <v>261</v>
       </c>
@@ -3675,9 +3675,9 @@
       <c r="E130" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F130" s="10"/>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F130" s="11"/>
+    </row>
+    <row r="131" spans="1:6">
       <c r="A131" s="2"/>
       <c r="B131" s="2" t="s">
         <v>138</v>
@@ -3691,9 +3691,9 @@
       <c r="E131" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F131" s="10"/>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F131" s="11"/>
+    </row>
+    <row r="132" spans="1:6">
       <c r="A132" s="2"/>
       <c r="B132" s="2" t="s">
         <v>140</v>
@@ -3707,9 +3707,9 @@
       <c r="E132" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="F132" s="10"/>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F132" s="11"/>
+    </row>
+    <row r="133" spans="1:6">
       <c r="A133" s="2"/>
       <c r="B133" s="2" t="s">
         <v>142</v>
@@ -3723,9 +3723,9 @@
       <c r="E133" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="F133" s="10"/>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F133" s="11"/>
+    </row>
+    <row r="134" spans="1:6">
       <c r="A134" s="2"/>
       <c r="B134" s="2" t="s">
         <v>144</v>
@@ -3739,9 +3739,9 @@
       <c r="E134" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F134" s="10"/>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F134" s="11"/>
+    </row>
+    <row r="135" spans="1:6">
       <c r="A135" s="2"/>
       <c r="B135" s="2" t="s">
         <v>101</v>
@@ -3755,9 +3755,9 @@
       <c r="E135" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F135" s="10"/>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F135" s="11"/>
+    </row>
+    <row r="136" spans="1:6">
       <c r="A136" s="2"/>
       <c r="B136" s="2" t="s">
         <v>146</v>
@@ -3771,9 +3771,9 @@
       <c r="E136" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="F136" s="10"/>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F136" s="11"/>
+    </row>
+    <row r="137" spans="1:6">
       <c r="A137" s="2"/>
       <c r="B137" s="2" t="s">
         <v>148</v>
@@ -3787,9 +3787,9 @@
       <c r="E137" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="F137" s="10"/>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F137" s="11"/>
+    </row>
+    <row r="138" spans="1:6">
       <c r="A138" s="2"/>
       <c r="B138" s="2" t="s">
         <v>150</v>
@@ -3803,9 +3803,9 @@
       <c r="E138" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="F138" s="10"/>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F138" s="11"/>
+    </row>
+    <row r="139" spans="1:6">
       <c r="A139" s="2"/>
       <c r="B139" s="2" t="s">
         <v>152</v>
@@ -3819,9 +3819,9 @@
       <c r="E139" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="F139" s="10"/>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F139" s="11"/>
+    </row>
+    <row r="140" spans="1:6">
       <c r="A140" s="2"/>
       <c r="B140" s="2" t="s">
         <v>154</v>
@@ -3835,9 +3835,9 @@
       <c r="E140" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="F140" s="10"/>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F140" s="11"/>
+    </row>
+    <row r="141" spans="1:6">
       <c r="A141" s="2"/>
       <c r="B141" s="2" t="s">
         <v>157</v>
@@ -3851,9 +3851,9 @@
       <c r="E141" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="F141" s="10"/>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F141" s="11"/>
+    </row>
+    <row r="142" spans="1:6">
       <c r="A142" s="2"/>
       <c r="B142" s="2" t="s">
         <v>159</v>
@@ -3865,9 +3865,9 @@
         <v>160</v>
       </c>
       <c r="E142" s="2"/>
-      <c r="F142" s="10"/>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F142" s="11"/>
+    </row>
+    <row r="143" spans="1:6">
       <c r="A143" s="3" t="s">
         <v>162</v>
       </c>
@@ -3883,9 +3883,9 @@
       <c r="E143" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F143" s="10"/>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F143" s="11"/>
+    </row>
+    <row r="144" spans="1:6">
       <c r="A144" s="2"/>
       <c r="B144" s="2" t="s">
         <v>300</v>
@@ -3899,9 +3899,9 @@
       <c r="E144" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F144" s="10"/>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F144" s="11"/>
+    </row>
+    <row r="145" spans="1:6">
       <c r="A145" s="2"/>
       <c r="B145" s="2" t="s">
         <v>164</v>
@@ -3915,9 +3915,9 @@
       <c r="E145" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F145" s="10"/>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F145" s="11"/>
+    </row>
+    <row r="146" spans="1:6">
       <c r="A146" s="2"/>
       <c r="B146" s="2" t="s">
         <v>166</v>
@@ -3931,9 +3931,9 @@
       <c r="E146" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F146" s="10"/>
-    </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F146" s="11"/>
+    </row>
+    <row r="147" spans="1:6">
       <c r="A147" s="2"/>
       <c r="B147" s="2" t="s">
         <v>168</v>
@@ -3945,9 +3945,9 @@
         <v>170</v>
       </c>
       <c r="E147" s="2"/>
-      <c r="F147" s="10"/>
-    </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F147" s="11"/>
+    </row>
+    <row r="148" spans="1:6">
       <c r="A148" s="2"/>
       <c r="B148" s="2" t="s">
         <v>171</v>
@@ -3959,9 +3959,9 @@
         <v>172</v>
       </c>
       <c r="E148" s="2"/>
-      <c r="F148" s="10"/>
-    </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F148" s="11"/>
+    </row>
+    <row r="149" spans="1:6">
       <c r="A149" s="2"/>
       <c r="B149" s="2" t="s">
         <v>173</v>
@@ -3973,9 +3973,9 @@
         <v>174</v>
       </c>
       <c r="E149" s="2"/>
-      <c r="F149" s="10"/>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F149" s="11"/>
+    </row>
+    <row r="150" spans="1:6">
       <c r="A150" s="2"/>
       <c r="B150" s="2" t="s">
         <v>305</v>
@@ -3987,9 +3987,9 @@
         <v>175</v>
       </c>
       <c r="E150" s="2"/>
-      <c r="F150" s="10"/>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F150" s="11"/>
+    </row>
+    <row r="151" spans="1:6">
       <c r="A151" s="2"/>
       <c r="B151" s="2" t="s">
         <v>176</v>
@@ -4001,9 +4001,9 @@
         <v>177</v>
       </c>
       <c r="E151" s="2"/>
-      <c r="F151" s="10"/>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F151" s="11"/>
+    </row>
+    <row r="152" spans="1:6">
       <c r="A152" s="2"/>
       <c r="B152" s="2" t="s">
         <v>178</v>
@@ -4015,9 +4015,9 @@
         <v>179</v>
       </c>
       <c r="E152" s="2"/>
-      <c r="F152" s="10"/>
-    </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F152" s="11"/>
+    </row>
+    <row r="153" spans="1:6">
       <c r="A153" s="2"/>
       <c r="B153" s="2" t="s">
         <v>306</v>
@@ -4029,9 +4029,9 @@
         <v>180</v>
       </c>
       <c r="E153" s="2"/>
-      <c r="F153" s="10"/>
-    </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F153" s="11"/>
+    </row>
+    <row r="154" spans="1:6">
       <c r="A154" s="2"/>
       <c r="B154" s="2" t="s">
         <v>181</v>
@@ -4043,9 +4043,9 @@
         <v>182</v>
       </c>
       <c r="E154" s="2"/>
-      <c r="F154" s="10"/>
-    </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F154" s="11"/>
+    </row>
+    <row r="155" spans="1:6">
       <c r="A155" s="2"/>
       <c r="B155" s="2" t="s">
         <v>183</v>
@@ -4057,9 +4057,9 @@
         <v>184</v>
       </c>
       <c r="E155" s="2"/>
-      <c r="F155" s="10"/>
-    </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F155" s="11"/>
+    </row>
+    <row r="156" spans="1:6">
       <c r="A156" s="2"/>
       <c r="B156" s="2" t="s">
         <v>185</v>
@@ -4071,9 +4071,9 @@
         <v>186</v>
       </c>
       <c r="E156" s="2"/>
-      <c r="F156" s="10"/>
-    </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F156" s="11"/>
+    </row>
+    <row r="157" spans="1:6">
       <c r="A157" s="3" t="s">
         <v>187</v>
       </c>
@@ -4089,9 +4089,9 @@
       <c r="E157" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F157" s="10"/>
-    </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F157" s="11"/>
+    </row>
+    <row r="158" spans="1:6">
       <c r="A158" s="3"/>
       <c r="B158" s="2" t="s">
         <v>65</v>
@@ -4106,7 +4106,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="159" spans="1:6">
       <c r="A159" s="3"/>
       <c r="B159" s="2" t="s">
         <v>74</v>
@@ -4121,7 +4121,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="160" spans="1:6">
       <c r="A160" s="2"/>
       <c r="B160" s="2" t="s">
         <v>5</v>
@@ -4136,7 +4136,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="161" spans="1:6">
       <c r="A161" s="2"/>
       <c r="B161" s="2" t="s">
         <v>281</v>
@@ -4151,7 +4151,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="162" spans="1:6">
       <c r="A162" s="2"/>
       <c r="B162" s="2" t="s">
         <v>280</v>
@@ -4166,7 +4166,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="163" spans="1:6">
       <c r="A163" s="2"/>
       <c r="B163" s="2" t="s">
         <v>190</v>
@@ -4181,7 +4181,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="164" spans="1:6">
       <c r="A164" s="2"/>
       <c r="B164" s="2" t="s">
         <v>194</v>
@@ -4196,7 +4196,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="165" spans="1:6">
       <c r="A165" s="2"/>
       <c r="B165" s="2" t="s">
         <v>28</v>
@@ -4211,7 +4211,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="166" spans="1:6">
       <c r="A166" s="2"/>
       <c r="B166" s="2" t="s">
         <v>30</v>
@@ -4224,7 +4224,7 @@
       </c>
       <c r="E166" s="2"/>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="167" spans="1:6">
       <c r="A167" s="3" t="s">
         <v>262</v>
       </c>
@@ -4241,7 +4241,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="168" spans="1:6">
       <c r="A168" s="2"/>
       <c r="B168" s="2" t="s">
         <v>197</v>
@@ -4256,7 +4256,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="169" spans="1:6">
       <c r="A169" s="2"/>
       <c r="B169" s="2" t="s">
         <v>161</v>
@@ -4271,7 +4271,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="170" spans="1:6">
       <c r="A170" s="2"/>
       <c r="B170" s="2" t="s">
         <v>279</v>
@@ -4286,7 +4286,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="171" spans="1:6">
       <c r="A171" s="2"/>
       <c r="B171" s="2" t="s">
         <v>200</v>
@@ -4301,7 +4301,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="172" spans="1:6">
       <c r="A172" s="2"/>
       <c r="B172" s="2" t="s">
         <v>202</v>
@@ -4316,7 +4316,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="173" spans="1:6">
       <c r="A173" s="2"/>
       <c r="B173" s="2" t="s">
         <v>204</v>
@@ -4331,7 +4331,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="174" spans="1:6">
       <c r="A174" s="2"/>
       <c r="B174" s="2" t="s">
         <v>206</v>
@@ -4346,7 +4346,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="175" spans="1:6">
       <c r="A175" s="2"/>
       <c r="B175" s="2" t="s">
         <v>208</v>
@@ -4361,7 +4361,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="176" spans="1:6">
       <c r="A176" s="3" t="s">
         <v>263</v>
       </c>
@@ -4377,11 +4377,11 @@
       <c r="E176" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F176" s="10" t="s">
+      <c r="F176" s="11" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="177" spans="1:6">
       <c r="A177" s="2"/>
       <c r="B177" s="2" t="s">
         <v>210</v>
@@ -4395,9 +4395,9 @@
       <c r="E177" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F177" s="10"/>
-    </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F177" s="11"/>
+    </row>
+    <row r="178" spans="1:6">
       <c r="A178" s="2"/>
       <c r="B178" s="2" t="s">
         <v>138</v>
@@ -4411,9 +4411,9 @@
       <c r="E178" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F178" s="10"/>
-    </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F178" s="11"/>
+    </row>
+    <row r="179" spans="1:6">
       <c r="A179" s="2"/>
       <c r="B179" s="2" t="s">
         <v>211</v>
@@ -4427,9 +4427,9 @@
       <c r="E179" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F179" s="10"/>
-    </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F179" s="11"/>
+    </row>
+    <row r="180" spans="1:6">
       <c r="A180" s="2"/>
       <c r="B180" s="2" t="s">
         <v>101</v>
@@ -4441,9 +4441,9 @@
         <v>346</v>
       </c>
       <c r="E180" s="2"/>
-      <c r="F180" s="10"/>
-    </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F180" s="11"/>
+    </row>
+    <row r="181" spans="1:6">
       <c r="A181" s="2"/>
       <c r="B181" s="2" t="s">
         <v>200</v>
@@ -4457,9 +4457,9 @@
       <c r="E181" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="F181" s="10"/>
-    </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F181" s="11"/>
+    </row>
+    <row r="182" spans="1:6">
       <c r="A182" s="2"/>
       <c r="B182" s="2" t="s">
         <v>202</v>
@@ -4471,9 +4471,9 @@
         <v>203</v>
       </c>
       <c r="E182" s="2"/>
-      <c r="F182" s="10"/>
-    </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F182" s="11"/>
+    </row>
+    <row r="183" spans="1:6">
       <c r="A183" s="2"/>
       <c r="B183" s="2" t="s">
         <v>204</v>
@@ -4485,9 +4485,9 @@
         <v>205</v>
       </c>
       <c r="E183" s="2"/>
-      <c r="F183" s="10"/>
-    </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F183" s="11"/>
+    </row>
+    <row r="184" spans="1:6">
       <c r="A184" s="2"/>
       <c r="B184" s="2" t="s">
         <v>206</v>
@@ -4499,9 +4499,9 @@
         <v>207</v>
       </c>
       <c r="E184" s="2"/>
-      <c r="F184" s="10"/>
-    </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="F184" s="11"/>
+    </row>
+    <row r="185" spans="1:6">
       <c r="A185" s="2"/>
       <c r="B185" s="2" t="s">
         <v>208</v>
@@ -4513,17 +4513,17 @@
         <v>209</v>
       </c>
       <c r="E185" s="2"/>
-      <c r="F185" s="10"/>
-    </row>
-    <row r="187" spans="1:6" ht="29.25" x14ac:dyDescent="0.8">
-      <c r="A187" s="8" t="s">
+      <c r="F185" s="11"/>
+    </row>
+    <row r="187" spans="1:6" ht="29.25">
+      <c r="A187" s="9" t="s">
         <v>352</v>
       </c>
-      <c r="B187" s="8"/>
-      <c r="C187" s="8"/>
-      <c r="D187" s="8"/>
-    </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.65">
+      <c r="B187" s="9"/>
+      <c r="C187" s="9"/>
+      <c r="D187" s="9"/>
+    </row>
+    <row r="188" spans="1:6">
       <c r="A188" s="4" t="s">
         <v>0</v>
       </c>
@@ -4540,7 +4540,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="189" spans="1:6">
       <c r="A189" s="3" t="s">
         <v>213</v>
       </c>
@@ -4557,7 +4557,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="190" spans="1:6">
       <c r="A190" s="2"/>
       <c r="B190" s="2" t="s">
         <v>5</v>
@@ -4572,7 +4572,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="191" spans="1:6">
       <c r="A191" s="2"/>
       <c r="B191" s="2" t="s">
         <v>345</v>
@@ -4587,7 +4587,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.65">
+    <row r="192" spans="1:6">
       <c r="A192" s="2"/>
       <c r="B192" s="2" t="s">
         <v>256</v>
@@ -4602,7 +4602,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="193" spans="1:5">
       <c r="A193" s="2"/>
       <c r="B193" s="2" t="s">
         <v>68</v>
@@ -4617,7 +4617,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="194" spans="1:5">
       <c r="A194" s="2"/>
       <c r="B194" s="2" t="s">
         <v>70</v>
@@ -4630,7 +4630,7 @@
       </c>
       <c r="E194" s="2"/>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="195" spans="1:5">
       <c r="A195" s="2"/>
       <c r="B195" s="2" t="s">
         <v>72</v>
@@ -4645,7 +4645,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="196" spans="1:5">
       <c r="A196" s="2"/>
       <c r="B196" s="2" t="s">
         <v>318</v>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="E196" s="2"/>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="197" spans="1:5">
       <c r="A197" s="2"/>
       <c r="B197" s="2" t="s">
         <v>28</v>
@@ -4673,7 +4673,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="198" spans="1:5">
       <c r="A198" s="2"/>
       <c r="B198" s="2" t="s">
         <v>30</v>
@@ -4688,7 +4688,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="199" spans="1:5">
       <c r="A199" s="3" t="s">
         <v>217</v>
       </c>
@@ -4705,7 +4705,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="200" spans="1:5">
       <c r="A200" s="2"/>
       <c r="B200" s="2" t="s">
         <v>5</v>
@@ -4720,7 +4720,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="201" spans="1:5">
       <c r="A201" s="2"/>
       <c r="B201" s="2" t="s">
         <v>345</v>
@@ -4735,7 +4735,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="202" spans="1:5">
       <c r="A202" s="2"/>
       <c r="B202" s="2" t="s">
         <v>256</v>
@@ -4750,7 +4750,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="203" spans="1:5">
       <c r="A203" s="2"/>
       <c r="B203" s="2" t="s">
         <v>68</v>
@@ -4765,7 +4765,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="204" spans="1:5">
       <c r="A204" s="2"/>
       <c r="B204" s="2" t="s">
         <v>70</v>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="E204" s="2"/>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="205" spans="1:5">
       <c r="A205" s="2"/>
       <c r="B205" s="2" t="s">
         <v>72</v>
@@ -4793,7 +4793,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="206" spans="1:5">
       <c r="A206" s="2"/>
       <c r="B206" s="2" t="s">
         <v>318</v>
@@ -4806,7 +4806,7 @@
       </c>
       <c r="E206" s="2"/>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="207" spans="1:5">
       <c r="A207" s="2"/>
       <c r="B207" s="2" t="s">
         <v>28</v>
@@ -4821,7 +4821,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="208" spans="1:5">
       <c r="A208" s="2"/>
       <c r="B208" s="2" t="s">
         <v>30</v>
@@ -4836,7 +4836,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="209" spans="1:5">
       <c r="A209" s="3" t="s">
         <v>219</v>
       </c>
@@ -4853,7 +4853,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="210" spans="1:5">
       <c r="A210" s="2"/>
       <c r="B210" s="2" t="s">
         <v>5</v>
@@ -4868,7 +4868,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="211" spans="1:5">
       <c r="A211" s="2"/>
       <c r="B211" s="2" t="s">
         <v>345</v>
@@ -4883,7 +4883,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="212" spans="1:5">
       <c r="A212" s="2"/>
       <c r="B212" s="2" t="s">
         <v>256</v>
@@ -4898,7 +4898,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="213" spans="1:5">
       <c r="A213" s="2"/>
       <c r="B213" s="2" t="s">
         <v>68</v>
@@ -4913,7 +4913,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="214" spans="1:5">
       <c r="A214" s="2"/>
       <c r="B214" s="2" t="s">
         <v>70</v>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="E214" s="2"/>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="215" spans="1:5">
       <c r="A215" s="6"/>
       <c r="B215" s="6" t="s">
         <v>221</v>
@@ -4941,7 +4941,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="216" spans="1:5">
       <c r="A216" s="2"/>
       <c r="B216" s="2" t="s">
         <v>72</v>
@@ -4956,7 +4956,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="217" spans="1:5">
       <c r="A217" s="2"/>
       <c r="B217" s="2" t="s">
         <v>28</v>
@@ -4971,7 +4971,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="218" spans="1:5">
       <c r="A218" s="2"/>
       <c r="B218" s="2" t="s">
         <v>30</v>
@@ -4986,7 +4986,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="219" spans="1:5">
       <c r="A219" s="3" t="s">
         <v>302</v>
       </c>
@@ -5003,7 +5003,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="220" spans="1:5">
       <c r="A220" s="2"/>
       <c r="B220" s="2" t="s">
         <v>76</v>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="E220" s="2"/>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="221" spans="1:5">
       <c r="A221" s="2"/>
       <c r="B221" s="2" t="s">
         <v>5</v>
@@ -5031,7 +5031,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="222" spans="1:5">
       <c r="A222" s="2"/>
       <c r="B222" s="2" t="s">
         <v>227</v>
@@ -5046,7 +5046,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="223" spans="1:5">
       <c r="A223" s="2"/>
       <c r="B223" s="2" t="s">
         <v>256</v>
@@ -5061,7 +5061,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="224" spans="1:5">
       <c r="A224" s="2"/>
       <c r="B224" s="2" t="s">
         <v>68</v>
@@ -5076,7 +5076,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="225" spans="1:5">
       <c r="A225" s="2"/>
       <c r="B225" s="2" t="s">
         <v>70</v>
@@ -5089,7 +5089,7 @@
       </c>
       <c r="E225" s="2"/>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="226" spans="1:5">
       <c r="A226" s="2"/>
       <c r="B226" s="2" t="s">
         <v>166</v>
@@ -5104,7 +5104,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="227" spans="1:5">
       <c r="A227" s="6"/>
       <c r="B227" s="6" t="s">
         <v>229</v>
@@ -5119,7 +5119,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="228" spans="1:5">
       <c r="A228" s="6"/>
       <c r="B228" s="6" t="s">
         <v>237</v>
@@ -5134,7 +5134,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="229" spans="1:5">
       <c r="A229" s="6"/>
       <c r="B229" s="6" t="s">
         <v>239</v>
@@ -5147,7 +5147,7 @@
       </c>
       <c r="E229" s="2"/>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="230" spans="1:5">
       <c r="A230" s="6"/>
       <c r="B230" s="6" t="s">
         <v>241</v>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="E230" s="2"/>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="231" spans="1:5">
       <c r="A231" s="6"/>
       <c r="B231" s="6" t="s">
         <v>332</v>
@@ -5173,7 +5173,7 @@
       </c>
       <c r="E231" s="2"/>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="232" spans="1:5">
       <c r="A232" s="6"/>
       <c r="B232" s="6" t="s">
         <v>231</v>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="E232" s="2"/>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="233" spans="1:5">
       <c r="A233" s="6"/>
       <c r="B233" s="6" t="s">
         <v>233</v>
@@ -5199,7 +5199,7 @@
       </c>
       <c r="E233" s="2"/>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="234" spans="1:5">
       <c r="A234" s="6"/>
       <c r="B234" s="6" t="s">
         <v>235</v>
@@ -5212,7 +5212,7 @@
       </c>
       <c r="E234" s="2"/>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="235" spans="1:5">
       <c r="A235" s="2"/>
       <c r="B235" s="2" t="s">
         <v>28</v>
@@ -5227,7 +5227,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="236" spans="1:5">
       <c r="A236" s="2"/>
       <c r="B236" s="2" t="s">
         <v>30</v>
@@ -5242,7 +5242,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="237" spans="1:5">
       <c r="A237" s="3" t="s">
         <v>334</v>
       </c>
@@ -5259,7 +5259,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="238" spans="1:5">
       <c r="A238" s="2"/>
       <c r="B238" s="2" t="s">
         <v>74</v>
@@ -5272,7 +5272,7 @@
       </c>
       <c r="E238" s="2"/>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="239" spans="1:5">
       <c r="A239" s="2"/>
       <c r="B239" s="2" t="s">
         <v>5</v>
@@ -5287,7 +5287,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="240" spans="1:5">
       <c r="A240" s="2"/>
       <c r="B240" s="2" t="s">
         <v>68</v>
@@ -5302,7 +5302,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="241" spans="1:5">
       <c r="A241" s="2"/>
       <c r="B241" s="2" t="s">
         <v>70</v>
@@ -5315,7 +5315,7 @@
       </c>
       <c r="E241" s="2"/>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="242" spans="1:5">
       <c r="A242" s="2"/>
       <c r="B242" s="2" t="s">
         <v>72</v>
@@ -5330,7 +5330,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="243" spans="1:5">
       <c r="A243" s="2"/>
       <c r="B243" s="2" t="s">
         <v>318</v>
@@ -5345,7 +5345,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="244" spans="1:5">
       <c r="A244" s="2"/>
       <c r="B244" s="2" t="s">
         <v>28</v>
@@ -5360,7 +5360,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.65">
+    <row r="245" spans="1:5">
       <c r="A245" s="2"/>
       <c r="B245" s="2" t="s">
         <v>30</v>
@@ -5375,19 +5375,19 @@
         <v>336</v>
       </c>
     </row>
-    <row r="247" spans="1:5" ht="117" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A247" s="11" t="s">
+    <row r="247" spans="1:5" ht="117" customHeight="1">
+      <c r="A247" s="8" t="s">
         <v>353</v>
       </c>
-      <c r="B247" s="11"/>
-      <c r="C247" s="11"/>
-      <c r="D247" s="11"/>
-      <c r="E247" s="11"/>
-    </row>
-    <row r="248" spans="1:5" ht="117" customHeight="1" x14ac:dyDescent="0.65"/>
-    <row r="249" spans="1:5" ht="117" customHeight="1" x14ac:dyDescent="0.65"/>
-    <row r="250" spans="1:5" ht="117" customHeight="1" x14ac:dyDescent="0.65"/>
-    <row r="251" spans="1:5" ht="117" customHeight="1" x14ac:dyDescent="0.65"/>
+      <c r="B247" s="8"/>
+      <c r="C247" s="8"/>
+      <c r="D247" s="8"/>
+      <c r="E247" s="8"/>
+    </row>
+    <row r="248" spans="1:5" ht="117" customHeight="1"/>
+    <row r="249" spans="1:5" ht="117" customHeight="1"/>
+    <row r="250" spans="1:5" ht="117" customHeight="1"/>
+    <row r="251" spans="1:5" ht="117" customHeight="1"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A247:E247"/>

</xml_diff>